<commit_message>
matlab pause between phases
</commit_message>
<xml_diff>
--- a/experiment/fMRI/scan_time_calculator.xlsx
+++ b/experiment/fMRI/scan_time_calculator.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c8b00b6d23712701/0. Tübingen Uni/Praktikum/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yavka\PycharmProjects\Arc-Rule-Generator\experiment\fMRI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C304404-B369-4EC4-A4E9-6BB5CD38E00B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D824E27D-F6F5-44AD-978D-A898F81C7F0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5190" yWindow="1643" windowWidth="16200" windowHeight="9307" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scan Time Calculator" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
     <t>Decision trials per block (inference + application)</t>
   </si>
   <si>
-    <t xml:space="preserve">Rest  between blocks (sec) </t>
+    <t xml:space="preserve">Rest between blocks (sec) </t>
   </si>
 </sst>
 </file>
@@ -409,34 +409,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="43.44140625" customWidth="1"/>
+    <col min="1" max="1" width="43.46484375" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -444,7 +444,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -452,49 +452,49 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>6</v>
       </c>
       <c r="B10">
         <f>5+B4</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>7</v>
       </c>
       <c r="B11">
         <f>2+B5</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>1</v>
       </c>
       <c r="B12">
         <f>((2+B5)*B6)+(B7)</f>
-        <v>250</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>2</v>
       </c>
       <c r="B14">
         <f>B10*B12</f>
-        <v>2250</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>3</v>
       </c>
       <c r="B15">
         <f>B14/60</f>
-        <v>37.5</v>
+        <v>17.333333333333332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
experiment scan time set
</commit_message>
<xml_diff>
--- a/experiment/fMRI/scan_time_calculator.xlsx
+++ b/experiment/fMRI/scan_time_calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yavka\PycharmProjects\Arc-Rule-Generator\experiment\fMRI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D824E27D-F6F5-44AD-978D-A898F81C7F0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458BCCBA-93C0-4EB9-AB2D-2DDE91FC4889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5190" yWindow="1643" windowWidth="16200" windowHeight="9307" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scan Time Calculator" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
     <t>Decision trials per block (inference + application)</t>
   </si>
   <si>
-    <t xml:space="preserve">Rest between blocks (sec) </t>
+    <t xml:space="preserve">Rest per blocks (middle &amp; end) </t>
   </si>
 </sst>
 </file>
@@ -425,7 +425,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
@@ -433,7 +433,7 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
@@ -449,7 +449,7 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
@@ -458,7 +458,7 @@
       </c>
       <c r="B10">
         <f>5+B4</f>
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
@@ -467,7 +467,7 @@
       </c>
       <c r="B11">
         <f>2+B5</f>
-        <v>10</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
@@ -476,7 +476,7 @@
       </c>
       <c r="B12">
         <f>((2+B5)*B6)+(B7)</f>
-        <v>130</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
@@ -485,7 +485,7 @@
       </c>
       <c r="B14">
         <f>B10*B12</f>
-        <v>1040</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
@@ -494,7 +494,7 @@
       </c>
       <c r="B15">
         <f>B14/60</f>
-        <v>17.333333333333332</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
excel scan time calculator updated
</commit_message>
<xml_diff>
--- a/experiment/fMRI/scan_time_calculator.xlsx
+++ b/experiment/fMRI/scan_time_calculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yavka\PycharmProjects\Arc-Rule-Generator\experiment\fMRI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yavuz Karaca\PycharmProjects\ArcRuleGenerator\experiment\fMRI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458BCCBA-93C0-4EB9-AB2D-2DDE91FC4889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BF659CD-49FB-4255-B271-AD44B35BC860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13044" yWindow="1236" windowWidth="15912" windowHeight="13644" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scan Time Calculator" sheetId="1" r:id="rId1"/>
@@ -33,43 +33,151 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
   <si>
     <t>fMRI Scan Time Calculator</t>
   </si>
   <si>
-    <t>Time per block (sec)</t>
-  </si>
-  <si>
-    <t>Total scan time (sec)</t>
-  </si>
-  <si>
-    <t>Total scan time (min)</t>
-  </si>
-  <si>
-    <t>Number of mixup blocks</t>
-  </si>
-  <si>
-    <t>Seconds per trial</t>
-  </si>
-  <si>
-    <t>Total blocks (5 family + mixup )</t>
-  </si>
-  <si>
-    <t>Trials per block (Bc +2 initial trials)</t>
-  </si>
-  <si>
-    <t>Decision trials per block (inference + application)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rest per blocks (middle &amp; end) </t>
+    <t>Rest time (sec)</t>
+  </si>
+  <si>
+    <t>Initial trial per phase</t>
+  </si>
+  <si>
+    <t>Total trials per phase</t>
+  </si>
+  <si>
+    <t>Total trials per block</t>
+  </si>
+  <si>
+    <t>Total rest per block (sec)</t>
+  </si>
+  <si>
+    <t>Total time per block (sec)</t>
+  </si>
+  <si>
+    <t>Fixed</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Legend:</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Phases </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>per block</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Decision trials</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> per phase</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Decision window</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> per trial</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (sec)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Blocks </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>per session</t>
+    </r>
+  </si>
+  <si>
+    <t>Total scan time  per session (sec)</t>
+  </si>
+  <si>
+    <t>Total scan time per session (min)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sessions </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>per subject</t>
+    </r>
+  </si>
+  <si>
+    <t>Current:</t>
+  </si>
+  <si>
+    <t>Total time per block (min)</t>
+  </si>
+  <si>
+    <t>My suggestion (6 decision trials, less sessions):</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -82,16 +190,51 @@
       <sz val="14"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF7F9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -99,19 +242,102 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFEBF7F9"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -408,94 +634,348 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.46484375" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="1" max="1" width="43.33203125" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="16">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="9"/>
+      <c r="B7" s="11"/>
+      <c r="D7" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="7">
         <v>4</v>
       </c>
-      <c r="B4">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="10">
+        <f>B8+B9</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="9"/>
+      <c r="B11" s="11"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="10">
+        <f>B12*B10</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="10">
+        <f>B6*2</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="10">
+        <f>(B5*B13)+B14</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="10">
+        <f>B15/60</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="9"/>
+      <c r="B17" s="11"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="13" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="B19" s="10">
+        <f>B18*B15</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="10">
+        <f>B19/60</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="9"/>
+      <c r="B21" s="11"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="7">
         <v>8</v>
       </c>
-      <c r="B5">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="10">
+        <f>B22*B19</f>
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="17">
+        <f>B23/60</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B29" s="16">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B30" s="7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="9"/>
+      <c r="B31" s="11"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32" s="7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34" s="10">
+        <f>B32+B33</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="9"/>
+      <c r="B35" s="11"/>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" s="10">
+        <f>B36*B34</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
+      <c r="B38" s="10">
+        <f>B30*2</f>
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B10">
-        <f>5+B4</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11">
-        <f>2+B5</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12">
-        <f>((2+B5)*B6)+(B7)</f>
-        <v>240</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B14">
-        <f>B10*B12</f>
+      <c r="B39" s="10">
+        <f>(B29*B37)+B38</f>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B40" s="10">
+        <f>B39/60</f>
+        <v>2.6666666666666665</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="9"/>
+      <c r="B41" s="11"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43" s="10">
+        <f>B42*B39</f>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B44" s="10">
+        <f>B43/60</f>
+        <v>13.333333333333334</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="9"/>
+      <c r="B45" s="11"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B46" s="7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="10">
+        <f>B46*B43</f>
         <v>4800</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15">
-        <f>B14/60</f>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B48" s="17">
+        <f>B47/60</f>
         <v>80</v>
       </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Scan time calculator updated for new design
</commit_message>
<xml_diff>
--- a/experiment/fMRI/scan_time_calculator.xlsx
+++ b/experiment/fMRI/scan_time_calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yavuz Karaca\PycharmProjects\ArcRuleGenerator\experiment\fMRI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBCDA4A3-44E9-46C4-A7E4-ED4128260E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6AAFC4A-507D-4E31-B0B2-467F326E8DDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13044" yWindow="1236" windowWidth="15912" windowHeight="13644" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10596" yWindow="1200" windowWidth="15912" windowHeight="13644" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scan Time Calculator" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
     <t>fMRI Scan Time Calculator</t>
   </si>
@@ -164,19 +164,44 @@
     </r>
   </si>
   <si>
-    <t>Current:</t>
-  </si>
-  <si>
     <t>Total time per block (min)</t>
   </si>
   <si>
-    <t>My suggestion (6 decision trials, less sessions):</t>
-  </si>
-  <si>
     <t>Total scan time  per subject (sec)</t>
   </si>
   <si>
     <t>Total scan time per subject (min)</t>
+  </si>
+  <si>
+    <t>Old:</t>
+  </si>
+  <si>
+    <t>Current Design:</t>
+  </si>
+  <si>
+    <r>
+      <t>Decision trials</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> per block</t>
+    </r>
+  </si>
+  <si>
+    <t>Initial trial per block</t>
+  </si>
+  <si>
+    <t>Rest time per block (sec)</t>
+  </si>
+  <si>
+    <t>Note: each block has rest at start, so at the end we have one additional rest</t>
   </si>
 </sst>
 </file>
@@ -640,11 +665,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="43.33203125" customWidth="1"/>
     <col min="2" max="2" width="9.109375" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
@@ -654,7 +680,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -755,7 +781,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16" s="10">
         <f>B15/60</f>
@@ -806,7 +832,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B23" s="10">
         <f>B22*B19</f>
@@ -815,7 +841,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B24" s="17">
         <f>B23/60</f>
@@ -824,7 +850,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
@@ -832,156 +858,129 @@
         <v>13</v>
       </c>
       <c r="B29" s="16">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B30" s="7">
-        <v>9</v>
-      </c>
+      <c r="A30" s="9"/>
+      <c r="B30" s="11"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="9"/>
-      <c r="B31" s="11"/>
+      <c r="A31" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="7">
+        <v>8</v>
+      </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="B32" s="7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B33" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="13" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B34" s="10">
-        <f>B32+B33</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="9"/>
-      <c r="B35" s="11"/>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B36" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B37" s="10">
-        <f>B36*B34</f>
+        <f>B31+B33</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B35" s="10">
+        <f>(B34*B29)+B32</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36" s="10">
+        <f>B35/60</f>
+        <v>1.6666666666666667</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="9"/>
+      <c r="B37" s="11"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="12" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="13" t="s">
+      <c r="B38" s="8">
         <v>5</v>
       </c>
-      <c r="B38" s="10">
-        <f>B30*2</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="13" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B39" s="10">
-        <f>(B29*B37)+B38</f>
-        <v>144</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+        <f>B38*B35</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B40" s="10">
         <f>B39/60</f>
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+        <v>8.3333333333333339</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="9"/>
       <c r="B41" s="11"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B42" s="7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="13" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B43" s="10">
-        <f>B42*B39</f>
-        <v>720</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B44" s="10">
+        <f>(B42*B39)+B32</f>
+        <v>4010</v>
+      </c>
+      <c r="D43" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B44" s="17">
         <f>B43/60</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" s="9"/>
-      <c r="B45" s="11"/>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B46" s="7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B47" s="10">
-        <f>B46*B43</f>
-        <v>4320</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="B48" s="17">
-        <f>B47/60</f>
-        <v>72</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A56" s="5"/>
+        <v>66.833333333333329</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Scan time table simplified
</commit_message>
<xml_diff>
--- a/experiment/fMRI/scan_time_calculator.xlsx
+++ b/experiment/fMRI/scan_time_calculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yavka\PycharmProjects\Arc-Rule-Generator\experiment\fMRI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yavuz Karaca\PycharmProjects\ArcRuleGenerator\experiment\fMRI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B117F9E-22DF-405F-85ED-3ADEDF34D631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6484B51-D801-42F8-8F13-6B9054376D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10596" yWindow="1200" windowWidth="15912" windowHeight="13644" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scan Time Calculator" sheetId="1" r:id="rId1"/>
@@ -33,26 +33,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>fMRI Scan Time Calculator</t>
   </si>
   <si>
-    <t>Rest time (sec)</t>
-  </si>
-  <si>
-    <t>Initial trial per phase</t>
-  </si>
-  <si>
-    <t>Total trials per phase</t>
-  </si>
-  <si>
     <t>Total trials per block</t>
   </si>
   <si>
-    <t>Total rest per block (sec)</t>
-  </si>
-  <si>
     <t>Total time per block (sec)</t>
   </si>
   <si>
@@ -66,38 +54,6 @@
   </si>
   <si>
     <t>Legend:</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Phases </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>per block</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Decision trials</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> per phase</t>
-    </r>
   </si>
   <si>
     <r>
@@ -164,19 +120,7 @@
     </r>
   </si>
   <si>
-    <t>Total time per block (min)</t>
-  </si>
-  <si>
-    <t>Total scan time  per subject (sec)</t>
-  </si>
-  <si>
     <t>Total scan time per subject (min)</t>
-  </si>
-  <si>
-    <t>Old:</t>
-  </si>
-  <si>
-    <t>Current Design:</t>
   </si>
   <si>
     <r>
@@ -201,9 +145,6 @@
     <t>Rest time per block (sec)</t>
   </si>
   <si>
-    <t>Total scan time per subject (sec)</t>
-  </si>
-  <si>
     <t>Includes one extra final rest and dummy triggers.</t>
   </si>
 </sst>
@@ -211,7 +152,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -226,15 +167,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -348,7 +280,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
@@ -361,6 +292,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -668,318 +600,137 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.33203125" customWidth="1"/>
-    <col min="2" max="2" width="9.1328125" customWidth="1"/>
-    <col min="4" max="4" width="21.46484375" customWidth="1"/>
+    <col min="1" max="1" width="36.77734375" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A4" s="5" t="s">
-        <v>22</v>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="15">
+        <v>10</v>
       </c>
       <c r="D4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="8"/>
+      <c r="B5" s="10"/>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="6">
+        <v>8</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="6">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A5" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="16">
+      <c r="D7" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="9">
+        <f>B6+B8</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="9">
+        <f>(B9*B4)+B7</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="8"/>
+      <c r="B11" s="10"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9">
+        <f>(B12*B10)+ (B7*2)</f>
+        <v>520</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A6" s="9"/>
-      <c r="B6" s="11"/>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A7" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="7">
-        <v>8</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A8" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="7">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A9" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A10" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="10">
-        <f>B7+B9</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A11" s="13" t="s">
+      <c r="B14" s="17">
+        <f>B13/60</f>
+        <v>8.6666666666666661</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="8"/>
+      <c r="B15" s="10"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="6">
         <v>6</v>
       </c>
-      <c r="B11" s="10">
-        <f>(B10*B5)+B8</f>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A12" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="10">
-        <f>B11/60</f>
-        <v>1.6666666666666667</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A13" s="9"/>
-      <c r="B13" s="11"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A14" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A15" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="10">
-        <f>(B14*B11)+ (B8*2)</f>
-        <v>520</v>
-      </c>
-      <c r="D15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A16" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="10">
-        <f>B15/60</f>
-        <v>8.6666666666666661</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A17" s="9"/>
-      <c r="B17" s="11"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A18" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A19" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="10">
-        <f>B18*B15</f>
-        <v>4160</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A20" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="17">
-        <f>B19/60</f>
-        <v>69.333333333333329</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A25" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A26" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B26" s="16">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A27" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B27" s="7">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A28" s="9"/>
-      <c r="B28" s="11"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A29" s="6" t="s">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B29" s="7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A30" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B30" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A31" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="10">
-        <f>B29+B30</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A32" s="9"/>
-      <c r="B32" s="11"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A33" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B33" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A34" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B34" s="10">
-        <f>B33*B31</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A35" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="B35" s="10">
-        <f>B27*2</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A36" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B36" s="10">
-        <f>(B26*B34)+B35</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A37" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B37" s="10">
-        <f>B36/60</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A38" s="9"/>
-      <c r="B38" s="11"/>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A39" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B39" s="7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A40" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B40" s="10">
-        <f>B39*B36</f>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A41" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B41" s="10">
-        <f>B40/60</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A42" s="9"/>
-      <c r="B42" s="11"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A43" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B43" s="7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A44" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B44" s="10">
-        <f>B43*B40</f>
-        <v>4800</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A45" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B45" s="17">
-        <f>B44/60</f>
-        <v>80</v>
+      <c r="B17" s="16">
+        <f>(B16*B13)/60</f>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>